<commit_message>
Parallel Execution 80% Done
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\July10\Framework01\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3485EBF0-C54C-47AC-AA57-5588589692FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9ED44BA-F98D-4694-875D-2CD400252596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="41">
   <si>
     <t>S.No</t>
   </si>
@@ -45,9 +45,6 @@
     <t>yes</t>
   </si>
   <si>
-    <t>openBrowser</t>
-  </si>
-  <si>
     <t>navigate</t>
   </si>
   <si>
@@ -70,9 +67,6 @@
   </si>
   <si>
     <t>clear</t>
-  </si>
-  <si>
-    <t>closeBrowser</t>
   </si>
   <si>
     <t>click</t>
@@ -208,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -306,57 +300,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -365,12 +314,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -383,9 +326,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -669,7 +609,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="45.140625" customWidth="1"/>
@@ -679,19 +619,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -702,7 +642,9 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="D2" s="2"/>
       <c r="E2" s="3" t="s">
         <v>5</v>
@@ -716,9 +658,11 @@
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="E3" s="3" t="s">
         <v>5</v>
       </c>
@@ -728,13 +672,11 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>5</v>
@@ -745,11 +687,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>5</v>
@@ -760,14 +704,12 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D6" s="2"/>
       <c r="E6" s="3" t="s">
         <v>5</v>
       </c>
@@ -782,7 +724,9 @@
       <c r="C7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="E7" s="3" t="s">
         <v>5</v>
       </c>
@@ -792,13 +736,11 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>5</v>
@@ -809,11 +751,11 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>5</v>
@@ -839,11 +781,11 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>5</v>
@@ -856,10 +798,10 @@
       <c r="B12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="D12" s="2"/>
       <c r="E12" s="3" t="s">
         <v>5</v>
       </c>
@@ -871,8 +813,8 @@
       <c r="B13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>29</v>
+      <c r="C13" s="7" t="s">
+        <v>8</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="3" t="s">
@@ -884,12 +826,14 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" s="2"/>
       <c r="E14" s="3" t="s">
         <v>5</v>
       </c>
@@ -899,13 +843,11 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>31</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>5</v>
@@ -916,11 +858,11 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>5</v>
@@ -931,12 +873,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C17" s="2"/>
-      <c r="D17" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="3" t="s">
         <v>5</v>
       </c>
@@ -946,9 +886,11 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="2"/>
+        <v>6</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="D18" s="2"/>
       <c r="E18" s="3" t="s">
         <v>5</v>
@@ -959,12 +901,12 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="E19" s="3" t="s">
         <v>5</v>
       </c>
@@ -974,11 +916,11 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>5</v>
@@ -989,12 +931,12 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
         <v>38</v>
       </c>
+      <c r="C21" s="2">
+        <v>0</v>
+      </c>
+      <c r="D21" s="2"/>
       <c r="E21" s="3" t="s">
         <v>5</v>
       </c>
@@ -1004,12 +946,14 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="2">
-        <v>0</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="E22" s="3" t="s">
         <v>5</v>
       </c>
@@ -1018,46 +962,16 @@
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="3"/>
-    </row>
-    <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10">
-        <v>24</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="5" t="s">
-        <v>5</v>
-      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" display="https://qaplayground.com/practice/input-fields" xr:uid="{68B571D7-D1B9-41EE-9539-2E3F5C8C50F9}"/>
-    <hyperlink ref="C14" r:id="rId2" xr:uid="{8EE3D130-B2AE-43CC-A13A-ACC4B1E52588}"/>
-    <hyperlink ref="C19" r:id="rId3" display="https://testautomationpractice.blogspot.com/" xr:uid="{30A38E6A-FF4B-4910-9F18-10E31AE9DEEE}"/>
+    <hyperlink ref="C2" r:id="rId1" display="https://qaplayground.com/practice/input-fields" xr:uid="{68B571D7-D1B9-41EE-9539-2E3F5C8C50F9}"/>
+    <hyperlink ref="C13" r:id="rId2" xr:uid="{8EE3D130-B2AE-43CC-A13A-ACC4B1E52588}"/>
+    <hyperlink ref="C18" r:id="rId3" display="https://testautomationpractice.blogspot.com/" xr:uid="{30A38E6A-FF4B-4910-9F18-10E31AE9DEEE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>

</xml_diff>

<commit_message>
Retry Analyzer Done and Allure Report Generation Types Done and total 90% Done Allure Report.
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\July10\Framework01\src\main\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\July30\Hybrid-Automation-Framework\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9ED44BA-F98D-4694-875D-2CD400252596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2907000F-8C4B-4AC3-B64B-480CDF688F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Allure Report Configuration Done with Retry Analyzer
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\July30\Hybrid-Automation-Framework\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2907000F-8C4B-4AC3-B64B-480CDF688F60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8EC67E-B551-4FC3-BB6E-B4F08704B345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="795" yWindow="1935" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -147,7 +147,7 @@
     <t>web.qa.url</t>
   </si>
   <si>
-    <t>web.tap.url</t>
+    <t>web.tap.ur</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Screenshot Folder Structure with word Document
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/TestData.xlsx
+++ b/src/main/resources/testdata/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\July30\Hybrid-Automation-Framework\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8EC67E-B551-4FC3-BB6E-B4F08704B345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{805547D3-8D45-4233-915E-A6B267FCC04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="795" yWindow="1935" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -147,7 +147,7 @@
     <t>web.qa.url</t>
   </si>
   <si>
-    <t>web.tap.ur</t>
+    <t>web.tap.url</t>
   </si>
 </sst>
 </file>

</xml_diff>